<commit_message>
new feature My Profile - Host
</commit_message>
<xml_diff>
--- a/documents/defect_list.xlsx
+++ b/documents/defect_list.xlsx
@@ -1,13 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\2025-2026_HKII\thi_tay_nghe\Seoul Stay - Rental Housing Project\documents\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82BE7BE-C074-4481-B1B5-49933ED21343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +28,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -66,6 +75,153 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>321543</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>121227</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE98FE68-CC13-6049-605F-4A603DC1E05C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1" y="0"/>
+          <a:ext cx="10625860" cy="5645727"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9867</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>86322</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A39EF00-7894-3DD6-0B3E-CDA2CC0A6D7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2448267" cy="4277322"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>533730</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>57876</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{510A10EA-98B2-F584-1BD4-F5CA7840B884}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2362530" cy="5201376"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +486,40 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2C627F-64D6-480E-8087-6D345AC8E656}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0850C008-157E-4DB7-9244-6110DB564740}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B4162B-79D2-474B-882F-BED609645246}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Upgrade feature and interface My Profile function
</commit_message>
<xml_diff>
--- a/documents/defect_list.xlsx
+++ b/documents/defect_list.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\2025-2026_HKII\thi_tay_nghe\Seoul Stay - Rental Housing Project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82BE7BE-C074-4481-B1B5-49933ED21343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DDD199-CF48-4F83-B43E-B62856258B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -213,6 +216,153 @@
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="2362530" cy="5201376"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>429706</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>162586</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31CBBD19-F49D-C4BB-22C2-CE692C675013}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7744906" cy="4734586"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>38446</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>96619</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C18F9E6C-826F-B90D-21B7-0C43F97BCA9B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2476846" cy="9812119"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>57924</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>143320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31B39B5E-DFF9-BE1C-062D-D2E73AE6120A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="5544324" cy="3191320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -522,4 +672,34 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24DAB39-4D20-4F9F-9466-2F9C96EB3B67}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF031D6F-6959-41F0-B149-6080A7FFF08E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A51BC7-EB3F-4820-AD32-C3CE33EE1B2A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
display picture on host item management and add feature tab item picture, display all record in amenities, users, area, sort and search
</commit_message>
<xml_diff>
--- a/documents/defect_list.xlsx
+++ b/documents/defect_list.xlsx
@@ -8,18 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\2025-2026_HKII\thi_tay_nghe\Seoul Stay - Rental Housing Project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DDD199-CF48-4F83-B43E-B62856258B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04259189-05B7-4B2B-A689-7D4D18BE9B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
+    <sheet name="S1_DF_25" sheetId="26" r:id="rId2"/>
+    <sheet name="S1_DF_24" sheetId="25" r:id="rId3"/>
+    <sheet name="S1_DF_23" sheetId="24" r:id="rId4"/>
+    <sheet name="S1_DF_22" sheetId="23" r:id="rId5"/>
+    <sheet name="S1_DF_21" sheetId="22" r:id="rId6"/>
+    <sheet name="S1_DF_20" sheetId="21" r:id="rId7"/>
+    <sheet name="S1_DF_19" sheetId="20" r:id="rId8"/>
+    <sheet name="S1_DF_18" sheetId="19" r:id="rId9"/>
+    <sheet name="S1_DF_17" sheetId="18" r:id="rId10"/>
+    <sheet name="S1_DF_16" sheetId="17" r:id="rId11"/>
+    <sheet name="S1_DF_15" sheetId="16" r:id="rId12"/>
+    <sheet name="S1_DF_14" sheetId="15" r:id="rId13"/>
+    <sheet name="S1_DF_13" sheetId="14" r:id="rId14"/>
+    <sheet name="S1_DF_12" sheetId="13" r:id="rId15"/>
+    <sheet name="S1_DF_11" sheetId="12" r:id="rId16"/>
+    <sheet name="S1_DF_10" sheetId="11" r:id="rId17"/>
+    <sheet name="S1_DF_9" sheetId="2" r:id="rId18"/>
+    <sheet name="S1_DF_8" sheetId="3" r:id="rId19"/>
+    <sheet name="S1_DF_7" sheetId="4" r:id="rId20"/>
+    <sheet name="S1_DF_6" sheetId="5" r:id="rId21"/>
+    <sheet name="S1_DF_5" sheetId="6" r:id="rId22"/>
+    <sheet name="S1_DF_4" sheetId="7" r:id="rId23"/>
+    <sheet name="S1_DF_3" sheetId="8" r:id="rId24"/>
+    <sheet name="S1_DF_2" sheetId="9" r:id="rId25"/>
+    <sheet name="S1_DF_1" sheetId="10" r:id="rId26"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,6 +47,23 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>khi nhập quá nhiều ký tự</t>
+  </si>
+  <si>
+    <t>capacity cho nhập vượt biên trên</t>
+  </si>
+  <si>
+    <t>minimum cho nhập vượt mức maximum</t>
+  </si>
+  <si>
+    <t>minimum cho nhập vượt biên trên</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -85,6 +121,398 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>58264</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>124480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D46E261-8BFC-E146-50B2-25F8461482A2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7983064" cy="4696480"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>77317</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>181638</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18CE04A3-8E21-99BC-622F-D163C0608343}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8002117" cy="4753638"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>181426</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>48350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D331080B-D0A2-9BDD-EB66-46D01DADA4A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="3229426" cy="5191850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>191633</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>76875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4E7626B-CEEA-0346-7849-E99B00D50187}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="8116433" cy="4839375"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>430812</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>38398</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD660436-91D1-D4AF-30C3-4A04D7D1E539}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="15670812" cy="2133898"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>278135</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>67429</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29F9A731-32B3-FE83-5C13-AFE846441F3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13689335" cy="5401429"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>68641</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>19797</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{015B7511-8C6A-5557-9138-81DF26FD4FA1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="14089441" cy="5353797"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>1106</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>67322</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B7FD9E5-6FD7-0E73-497D-EDE5FAE50C49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7925906" cy="4639322"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>1</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -129,7 +557,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -178,7 +606,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -227,7 +655,56 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>553548</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57796</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4E1CB0A-F29E-E98C-5965-D8417BC39229}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7868748" cy="4629796"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing20.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -276,7 +753,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -325,7 +802,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing22.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -363,6 +840,540 @@
         <a:xfrm>
           <a:off x="0" y="0"/>
           <a:ext cx="5544324" cy="3191320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing23.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>116018</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>162586</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7BDEB729-6F18-7F66-17C9-31B6DFBE5E2A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12308018" cy="4734586"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing24.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>29430</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>181665</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2055854-7941-000C-6E73-44DBD05E464D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6125430" cy="4944165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing25.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>505491</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>95928</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34CE4231-8394-18A8-1F01-2453C3B370F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="4772691" cy="4858428"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>420094</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>47711</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B613BEE-8E95-3FBC-9C9E-315221AE650D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7125694" cy="619211"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>420094</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>47711</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C09CAA4-2E21-C8E9-1B77-620F9C34B370}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7125694" cy="619211"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>543426</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>115034</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{847AB4A9-585B-45DA-4D63-24DA21D715C0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="3591426" cy="5258534"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>601180</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>181638</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08DFECC8-749D-EDD4-493A-671727A9E178}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7916380" cy="4753638"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>601180</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>181638</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EB84FC0-DB5E-0A7B-B352-D9C5799D600B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7916380" cy="4753638"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>601180</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>181638</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3883592-48CA-1302-67C7-3F8A930DEBA0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7916380" cy="4753638"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>29685</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>76849</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE9AECB0-5F48-659B-0244-0173907DF48E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7954485" cy="4648849"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>305255</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>134060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C0B7842-B7C5-CE01-3F65-28979459141A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8020050" y="0"/>
+          <a:ext cx="3258005" cy="5087060"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -644,8 +1655,190 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BD3C64-69EB-4302-BD62-8D3A11B4E3E7}">
+  <dimension ref="D33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72FE168-9FC6-48CD-95CB-99E0C198C94D}">
+  <dimension ref="Q14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="14" spans="17:17" x14ac:dyDescent="0.25">
+      <c r="Q14" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44ADF79B-0E92-42F6-9FDC-3D2CE2236779}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B738F73-3317-4241-85FB-A56AD79F71AC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38FD7470-AAAD-4245-918C-4AF1956B374C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E2A768A-C4A5-4890-8F15-A8D707110F83}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81492F5D-90BC-451F-9786-44E76F657A18}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67E53937-ED0B-433D-A426-7644088A3F9C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2C627F-64D6-480E-8087-6D345AC8E656}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0850C008-157E-4DB7-9244-6110DB564740}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2C627F-64D6-480E-8087-6D345AC8E656}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E54157CA-BDA1-4D35-86B2-D592697DF60D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B4162B-79D2-474B-882F-BED609645246}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24DAB39-4D20-4F9F-9466-2F9C96EB3B67}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF031D6F-6959-41F0-B149-6080A7FFF08E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A51BC7-EB3F-4820-AD32-C3CE33EE1B2A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B52DE20B-C35E-4E6D-A887-04217B7E1070}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DEB1486-6A2C-48F0-9AAE-13D23F6697E9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DF64AD-212F-4F23-BD97-16E00A07E752}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -655,7 +1848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0850C008-157E-4DB7-9244-6110DB564740}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7A002F4-01C0-4643-89F6-DE12FA4FECEC}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -665,27 +1858,39 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B4162B-79D2-474B-882F-BED609645246}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705D94DE-8871-4581-8436-D5AC25E9214C}">
+  <dimension ref="C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="7" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24DAB39-4D20-4F9F-9466-2F9C96EB3B67}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA18EDFD-E9C6-4822-BD55-A0962D4B8F6C}">
+  <dimension ref="D9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF031D6F-6959-41F0-B149-6080A7FFF08E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C21D7208-9E67-4E99-9724-C18A88778C84}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -695,7 +1900,27 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3A51BC7-EB3F-4820-AD32-C3CE33EE1B2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAE80C34-4E57-4BA5-9E82-304576E8D993}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{919FA6FE-5862-4C72-B385-5FDE28306A4E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8DB91B8-6948-4306-9746-9DB3AA8B762F}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>